<commit_message>
Diet bulk grid: add Meal Type + Day columns
- Diet grid columns now: Day, Meal Type (Breakfast/Lunch/Dinner/Snack), Meal,
  Items, macros. Meal Type sets the client nutrition grouping directly (was
  inferred from the meal name); Day schedules the meal.
- AI import extracts day + mealType; round-trips through the meal-plan library.
- Client nutrition view shows a day badge per meal; Guided/Full 'today' meal
  subtitle shows day + type. Diet CSV/XLSX templates updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/diet-template.xlsx
+++ b/public/templates/diet-template.xlsx
@@ -397,159 +397,203 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>day</v>
+      </c>
+      <c r="B1" t="str">
+        <v>mealType</v>
+      </c>
+      <c r="C1" t="str">
         <v>meal</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
         <v>items</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>calories</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>protein</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>carbs</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>fat</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>High Carb — Meal 1</v>
+        <v>Monday</v>
       </c>
       <c r="B2" t="str">
+        <v>Breakfast</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Morning Smoothie + Eggs</v>
+      </c>
+      <c r="D2" t="str">
         <v>Medipure smoothie, 2 eggs, turkey bacon</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>520</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>32</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>45</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>High Carb — Meal 2</v>
+        <v>Monday</v>
       </c>
       <c r="B3" t="str">
+        <v>Lunch</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Power Bowl</v>
+      </c>
+      <c r="D3" t="str">
         <v>6oz sweet potato, 4oz turkey, asparagus, olive oil</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>610</v>
       </c>
-      <c r="D3">
+      <c r="F3">
         <v>40</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>60</v>
       </c>
-      <c r="F3">
+      <c r="H3">
         <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>High Carb — Meal 3</v>
+        <v>Monday</v>
       </c>
       <c r="B4" t="str">
+        <v>Dinner</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Fish Plate</v>
+      </c>
+      <c r="D4" t="str">
         <v>4oz salmon, quinoa, greens, olive oil</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>560</v>
       </c>
-      <c r="D4">
+      <c r="F4">
         <v>38</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>42</v>
       </c>
-      <c r="F4">
+      <c r="H4">
         <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Low Carb — Meal 1</v>
+        <v>Monday</v>
       </c>
       <c r="B5" t="str">
-        <v>2 eggs scrambled, spinach, pepper, Medipure shake</v>
-      </c>
-      <c r="C5">
-        <v>430</v>
-      </c>
-      <c r="D5">
-        <v>34</v>
+        <v>Snack</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Protein Shake</v>
+      </c>
+      <c r="D5" t="str">
+        <v>1 scoop protein, almond milk</v>
       </c>
       <c r="E5">
-        <v>10</v>
+        <v>180</v>
       </c>
       <c r="F5">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Low Carb — Meal 2</v>
+        <v>Tuesday</v>
       </c>
       <c r="B6" t="str">
-        <v>bone broth, 5oz beef, cauliflower rice, ghee</v>
-      </c>
-      <c r="C6">
-        <v>520</v>
-      </c>
-      <c r="D6">
-        <v>42</v>
+        <v>Breakfast</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Egg Scramble + Shake</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2 eggs, spinach, pepper, Medipure shake</v>
       </c>
       <c r="E6">
-        <v>12</v>
+        <v>430</v>
       </c>
       <c r="F6">
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Low Carb — Meal 3</v>
+        <v>Tuesday</v>
       </c>
       <c r="B7" t="str">
+        <v>Dinner</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Salmon Salad</v>
+      </c>
+      <c r="D7" t="str">
         <v>6oz salmon, arugula, avocado, olive oil + vinegar</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>540</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <v>44</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>8</v>
       </c>
-      <c r="F7">
+      <c r="H7">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>